<commit_message>
setor - bens basicos
</commit_message>
<xml_diff>
--- a/graficos_tabelas/preliminares/Tabela_resumo_thetas.xlsx
+++ b/graficos_tabelas/preliminares/Tabela_resumo_thetas.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6e8fc6e241c731ae/UFABC/Dissertação/volatilidade-IBOV-GPR/Impacto-geopolitico-ibovespa/graficos_tabelas/preliminares/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="575" documentId="11_F25DC773A252ABDACC1048C0F11B46C65ADE58EB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0412E99C-3BB9-4011-8056-68D0DCB2BDC1}"/>
+  <xr:revisionPtr revIDLastSave="654" documentId="11_F25DC773A252ABDACC1048C0F11B46C65ADE58EB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30B98A5B-EB48-4703-957F-A9EA5F3A3E90}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IBOV" sheetId="1" r:id="rId1"/>
     <sheet name="SETORES" sheetId="2" r:id="rId2"/>
     <sheet name="CONSUMO" sheetId="3" r:id="rId3"/>
+    <sheet name="BENS BASICOS" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="277">
   <si>
     <t>Garch-Midas nos retornos do Ibovespa</t>
   </si>
@@ -756,6 +757,108 @@
   </si>
   <si>
     <t>0.066</t>
+  </si>
+  <si>
+    <t>SETOR BENS BASICOS X CAMBIO</t>
+  </si>
+  <si>
+    <t>MODELO 2 - GPR GLOBAL E VAR CAMBIO ASSIMÉTRICO - SETOR: BENS BASICOS</t>
+  </si>
+  <si>
+    <t>0.1558</t>
+  </si>
+  <si>
+    <t>0.186</t>
+  </si>
+  <si>
+    <t>-0.1153</t>
+  </si>
+  <si>
+    <t>0.019</t>
+  </si>
+  <si>
+    <t>-0.1218</t>
+  </si>
+  <si>
+    <t>0.009</t>
+  </si>
+  <si>
+    <t>-0.4601</t>
+  </si>
+  <si>
+    <t>-0.3733</t>
+  </si>
+  <si>
+    <t>0.243</t>
+  </si>
+  <si>
+    <t>-0.2644</t>
+  </si>
+  <si>
+    <t>-0.0636</t>
+  </si>
+  <si>
+    <t>0.069</t>
+  </si>
+  <si>
+    <t>-0.6628</t>
+  </si>
+  <si>
+    <t>0.001</t>
+  </si>
+  <si>
+    <t>0.2691</t>
+  </si>
+  <si>
+    <t>-0.6661</t>
+  </si>
+  <si>
+    <t>0.003</t>
+  </si>
+  <si>
+    <t>-0.0843</t>
+  </si>
+  <si>
+    <t>0.143</t>
+  </si>
+  <si>
+    <t>-0.4793</t>
+  </si>
+  <si>
+    <t>-0.0974</t>
+  </si>
+  <si>
+    <t>0.106</t>
+  </si>
+  <si>
+    <t>-0.4883</t>
+  </si>
+  <si>
+    <t>0.054</t>
+  </si>
+  <si>
+    <t>-0.0956</t>
+  </si>
+  <si>
+    <t>0.086</t>
+  </si>
+  <si>
+    <t>-0.5405</t>
+  </si>
+  <si>
+    <t>-0.3608</t>
+  </si>
+  <si>
+    <t>0.088</t>
+  </si>
+  <si>
+    <t>-0.6781</t>
+  </si>
+  <si>
+    <t>-0.3974</t>
+  </si>
+  <si>
+    <t>0.205</t>
   </si>
 </sst>
 </file>
@@ -849,7 +952,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -865,6 +968,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3200,4 +3304,689 @@
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF7E7DD8-1A46-4903-B932-981461A1B017}">
+  <dimension ref="A1:J29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="4">
+        <v>-1190</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="1">
+        <v>12</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="1">
+        <v>12</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="1">
+        <v>6</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="1">
+        <v>6</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="I15" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="J15" s="9" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="1">
+        <v>3</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F16" s="1">
+        <v>3</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="I16" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="1">
+        <v>3</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F17" s="1">
+        <v>1</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="I17" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="1">
+        <v>12</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F18" s="1">
+        <v>12</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="J18" s="5" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="1">
+        <v>6</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F19" s="1">
+        <v>6</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="I19" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="J19" s="9" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="1">
+        <v>3</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F20" s="1">
+        <v>3</v>
+      </c>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" s="1">
+        <v>3</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F21" s="1">
+        <v>1</v>
+      </c>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="1">
+        <v>12</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F22" s="1">
+        <v>12</v>
+      </c>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="1">
+        <v>6</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F23" s="1">
+        <v>6</v>
+      </c>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="9"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="1">
+        <v>3</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F24" s="1">
+        <v>3</v>
+      </c>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="9"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25" s="1">
+        <v>3</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F25" s="1">
+        <v>1</v>
+      </c>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="9"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="1">
+        <v>12</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F26" s="1">
+        <v>12</v>
+      </c>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="9"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="1">
+        <v>6</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F27" s="1">
+        <v>6</v>
+      </c>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="9"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="1">
+        <v>3</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F28" s="1">
+        <v>3</v>
+      </c>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="9"/>
+      <c r="J28" s="9"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" s="1">
+        <v>3</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F29" s="1">
+        <v>1</v>
+      </c>
+      <c r="G29" s="9"/>
+      <c r="H29" s="9"/>
+      <c r="I29" s="9"/>
+      <c r="J29" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A6:I6"/>
+    <mergeCell ref="A12:J12"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
setor - bens basicos - cambio
</commit_message>
<xml_diff>
--- a/graficos_tabelas/preliminares/Tabela_resumo_thetas.xlsx
+++ b/graficos_tabelas/preliminares/Tabela_resumo_thetas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6e8fc6e241c731ae/UFABC/Dissertação/volatilidade-IBOV-GPR/Impacto-geopolitico-ibovespa/graficos_tabelas/preliminares/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="654" documentId="11_F25DC773A252ABDACC1048C0F11B46C65ADE58EB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30B98A5B-EB48-4703-957F-A9EA5F3A3E90}"/>
+  <xr:revisionPtr revIDLastSave="713" documentId="11_F25DC773A252ABDACC1048C0F11B46C65ADE58EB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D66360B2-ED2D-400F-8760-1D3321899FE1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="308">
   <si>
     <t>Garch-Midas nos retornos do Ibovespa</t>
   </si>
@@ -859,6 +859,99 @@
   </si>
   <si>
     <t>0.205</t>
+  </si>
+  <si>
+    <t>-0.4791</t>
+  </si>
+  <si>
+    <t>-0.2767</t>
+  </si>
+  <si>
+    <t>-0.5350</t>
+  </si>
+  <si>
+    <t>0.008</t>
+  </si>
+  <si>
+    <t>-0.0628</t>
+  </si>
+  <si>
+    <t>0.072</t>
+  </si>
+  <si>
+    <t>0.300</t>
+  </si>
+  <si>
+    <t>0.0083</t>
+  </si>
+  <si>
+    <t>0.087</t>
+  </si>
+  <si>
+    <t>-0.4346</t>
+  </si>
+  <si>
+    <t>0.482</t>
+  </si>
+  <si>
+    <t>-0.1174</t>
+  </si>
+  <si>
+    <t>0.029</t>
+  </si>
+  <si>
+    <t>-0.1203</t>
+  </si>
+  <si>
+    <t>0.387</t>
+  </si>
+  <si>
+    <t>-0.1288</t>
+  </si>
+  <si>
+    <t>-0.1205</t>
+  </si>
+  <si>
+    <t>0.365</t>
+  </si>
+  <si>
+    <t>0.007</t>
+  </si>
+  <si>
+    <t>0.244</t>
+  </si>
+  <si>
+    <t>-0.4669</t>
+  </si>
+  <si>
+    <t>-0.5964</t>
+  </si>
+  <si>
+    <t>-0.3770</t>
+  </si>
+  <si>
+    <t>0.245</t>
+  </si>
+  <si>
+    <t>-0.1554</t>
+  </si>
+  <si>
+    <t>0.343</t>
+  </si>
+  <si>
+    <t>-0.2732</t>
+  </si>
+  <si>
+    <t>0.4192</t>
+  </si>
+  <si>
+    <t>0.647</t>
+  </si>
+  <si>
+    <t>-0.0692</t>
+  </si>
+  <si>
+    <t>0.063</t>
   </si>
 </sst>
 </file>
@@ -968,7 +1061,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3568,13 +3663,13 @@
       <c r="F14" s="1">
         <v>12</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="1" t="s">
         <v>257</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="I14" s="9" t="s">
+      <c r="I14" s="1" t="s">
         <v>259</v>
       </c>
       <c r="J14" s="3" t="s">
@@ -3600,16 +3695,16 @@
       <c r="F15" s="1">
         <v>6</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="1" t="s">
         <v>260</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>261</v>
       </c>
-      <c r="I15" s="9" t="s">
+      <c r="I15" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="J15" s="9" t="s">
+      <c r="J15" s="1" t="s">
         <v>263</v>
       </c>
     </row>
@@ -3632,13 +3727,13 @@
       <c r="F16" s="1">
         <v>3</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="1" t="s">
         <v>264</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="I16" s="9" t="s">
+      <c r="I16" s="1" t="s">
         <v>265</v>
       </c>
       <c r="J16" s="5" t="s">
@@ -3664,13 +3759,13 @@
       <c r="F17" s="1">
         <v>1</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="1" t="s">
         <v>267</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="I17" s="9" t="s">
+      <c r="I17" s="1" t="s">
         <v>269</v>
       </c>
       <c r="J17" s="5" t="s">
@@ -3696,13 +3791,13 @@
       <c r="F18" s="1">
         <v>12</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="G18" s="1" t="s">
         <v>271</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="I18" s="9" t="s">
+      <c r="I18" s="1" t="s">
         <v>272</v>
       </c>
       <c r="J18" s="5" t="s">
@@ -3728,16 +3823,16 @@
       <c r="F19" s="1">
         <v>6</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="1" t="s">
         <v>274</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="I19" s="9" t="s">
+      <c r="I19" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="J19" s="9" t="s">
+      <c r="J19" s="1" t="s">
         <v>276</v>
       </c>
     </row>
@@ -3760,10 +3855,18 @@
       <c r="F20" s="1">
         <v>3</v>
       </c>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
+      <c r="G20" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
@@ -3784,10 +3887,18 @@
       <c r="F21" s="1">
         <v>1</v>
       </c>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
+      <c r="G21" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>282</v>
+      </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
@@ -3808,10 +3919,18 @@
       <c r="F22" s="1">
         <v>12</v>
       </c>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
+      <c r="G22" s="9">
+        <v>-1339</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="J22" s="5" t="s">
+        <v>285</v>
+      </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
@@ -3832,10 +3951,18 @@
       <c r="F23" s="1">
         <v>6</v>
       </c>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="9"/>
+      <c r="G23" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
@@ -3856,10 +3983,18 @@
       <c r="F24" s="1">
         <v>3</v>
       </c>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
+      <c r="G24" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
@@ -3880,10 +4015,18 @@
       <c r="F25" s="1">
         <v>1</v>
       </c>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
+      <c r="G25" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>295</v>
+      </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
@@ -3904,10 +4047,18 @@
       <c r="F26" s="1">
         <v>12</v>
       </c>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="9"/>
+      <c r="G26" s="9">
+        <v>-1519</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="J26" s="5" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
@@ -3928,10 +4079,18 @@
       <c r="F27" s="1">
         <v>6</v>
       </c>
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
+      <c r="G27" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>300</v>
+      </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
@@ -3952,10 +4111,18 @@
       <c r="F28" s="1">
         <v>3</v>
       </c>
-      <c r="G28" s="9"/>
-      <c r="H28" s="9"/>
-      <c r="I28" s="9"/>
-      <c r="J28" s="9"/>
+      <c r="G28" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
@@ -3976,10 +4143,18 @@
       <c r="F29" s="1">
         <v>1</v>
       </c>
-      <c r="G29" s="9"/>
-      <c r="H29" s="9"/>
-      <c r="I29" s="9"/>
-      <c r="J29" s="9"/>
+      <c r="G29" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="J29" s="5" t="s">
+        <v>307</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
descritivas - retornos e mensais
</commit_message>
<xml_diff>
--- a/graficos_tabelas/preliminares/Tabela_resumo_thetas.xlsx
+++ b/graficos_tabelas/preliminares/Tabela_resumo_thetas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6e8fc6e241c731ae/UFABC/Dissertação/volatilidade-IBOV-GPR/Impacto-geopolitico-ibovespa/graficos_tabelas/preliminares/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="713" documentId="11_F25DC773A252ABDACC1048C0F11B46C65ADE58EB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D66360B2-ED2D-400F-8760-1D3321899FE1}"/>
+  <xr:revisionPtr revIDLastSave="733" documentId="11_F25DC773A252ABDACC1048C0F11B46C65ADE58EB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8DF6CF67-1D4A-4C76-8214-2BB80FD9C855}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="316">
   <si>
     <t>Garch-Midas nos retornos do Ibovespa</t>
   </si>
@@ -111,9 +111,6 @@
     <t>-0.002</t>
   </si>
   <si>
-    <t>Não estacionário</t>
-  </si>
-  <si>
     <t>Estacionário</t>
   </si>
   <si>
@@ -952,6 +949,33 @@
   </si>
   <si>
     <t>0.063</t>
+  </si>
+  <si>
+    <t>0.404</t>
+  </si>
+  <si>
+    <t>0.275</t>
+  </si>
+  <si>
+    <t>0.500</t>
+  </si>
+  <si>
+    <t>-0.0035</t>
+  </si>
+  <si>
+    <t>0.202</t>
+  </si>
+  <si>
+    <t>-0.0046</t>
+  </si>
+  <si>
+    <t>0.082</t>
+  </si>
+  <si>
+    <t>-0.0013</t>
+  </si>
+  <si>
+    <t>0.226</t>
   </si>
 </sst>
 </file>
@@ -1348,7 +1372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -1498,7 +1522,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -1532,345 +1556,336 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>166</v>
+        <v>310</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>311</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>168</v>
+        <v>312</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>313</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>169</v>
+        <v>314</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>170</v>
+        <v>315</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="F15" s="1" t="s">
+      <c r="E16" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="G16" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="G15" s="5" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>4</v>
-      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B19" s="1">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>2</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F19" s="1">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J19" t="s">
-        <v>56</v>
-      </c>
-      <c r="K19" t="s">
-        <v>57</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>35</v>
+        <v>5</v>
+      </c>
+      <c r="B20" s="1">
+        <v>0</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>179</v>
+        <v>307</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>37</v>
+        <v>26</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="F20" s="1">
+        <v>0</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="H20" t="s">
-        <v>28</v>
-      </c>
-      <c r="J20" t="s">
-        <v>56</v>
-      </c>
-      <c r="K20" t="s">
-        <v>58</v>
+        <v>309</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>172</v>
+        <v>35</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>179</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="H21" t="s">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="J21" t="s">
+        <v>55</v>
+      </c>
+      <c r="K21" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="H22" t="s">
+        <v>27</v>
+      </c>
+      <c r="J22" t="s">
+        <v>55</v>
+      </c>
+      <c r="K22" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B23" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F23" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G22" s="3" t="s">
+      <c r="G23" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="6"/>
-    </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="K25" t="s">
-        <v>84</v>
-      </c>
+      <c r="A25" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="6"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C26" s="1">
-        <v>12</v>
+        <v>72</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>74</v>
       </c>
       <c r="D26" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="K26" t="s">
         <v>83</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F26" s="1">
-        <v>12</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="J26" s="3" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C27" s="1">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F27" s="1">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="H27" s="3" t="s">
-        <v>90</v>
+        <v>84</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>86</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C28" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F28" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>94</v>
+        <v>88</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>89</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>6</v>
@@ -1879,126 +1894,126 @@
         <v>3</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F29" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C30" s="1">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F30" s="1">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C31" s="1">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>7</v>
       </c>
       <c r="F31" s="1">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C32" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>7</v>
       </c>
       <c r="F32" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="J32" s="5" t="s">
-        <v>112</v>
+        <v>106</v>
+      </c>
+      <c r="J32" s="3" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>6</v>
@@ -2007,126 +2022,126 @@
         <v>3</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>7</v>
       </c>
       <c r="F33" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="J33" s="1" t="s">
-        <v>116</v>
+        <v>109</v>
+      </c>
+      <c r="J33" s="5" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C34" s="1">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F34" s="1">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="J34" s="3" t="s">
-        <v>120</v>
+        <v>113</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C35" s="1">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F35" s="1">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C36" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F36" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>96</v>
+        <v>123</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>7</v>
@@ -2135,126 +2150,126 @@
         <v>3</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F37" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>131</v>
+        <v>95</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C38" s="1">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F38" s="1">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>101</v>
+        <v>130</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C39" s="1">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>7</v>
       </c>
       <c r="F39" s="1">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>138</v>
+        <v>100</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C40" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>7</v>
       </c>
       <c r="F40" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>142</v>
+        <v>135</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>7</v>
@@ -2263,32 +2278,64 @@
         <v>3</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>7</v>
       </c>
       <c r="F41" s="1">
+        <v>3</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="J41" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="1">
+        <v>3</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F42" s="1">
         <v>1</v>
       </c>
-      <c r="G41" s="1" t="s">
+      <c r="G42" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="H42" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="I42" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="H41" s="5" t="s">
+      <c r="J42" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="I41" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J41" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A17:G17"/>
-    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A25:J25"/>
     <mergeCell ref="A12:G12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2308,22 +2355,22 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -2357,22 +2404,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>16</v>
@@ -2380,22 +2427,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>16</v>
@@ -2403,7 +2450,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -2437,53 +2484,53 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="G12" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>210</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -2517,22 +2564,22 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>10</v>
@@ -2540,7 +2587,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B19" s="4">
         <v>-1190</v>
@@ -2549,13 +2596,13 @@
         <v>16</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>16</v>
@@ -2563,7 +2610,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -2597,22 +2644,22 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G23" s="1" t="s">
         <v>16</v>
@@ -2620,22 +2667,22 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>16</v>
@@ -2671,7 +2718,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -2705,53 +2752,53 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="G3" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>210</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -2785,7 +2832,7 @@
         <v>4</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>4</v>
@@ -2793,36 +2840,36 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="G8" s="1" t="s">
-        <v>156</v>
-      </c>
       <c r="H8" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="I8" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -2835,7 +2882,7 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -2849,39 +2896,39 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C13" s="1" t="s">
+      <c r="D13" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="G13" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F13" s="1" t="s">
+      <c r="H13" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="I13" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="G13" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="H13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>6</v>
@@ -2890,7 +2937,7 @@
         <v>12</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>6</v>
@@ -2899,21 +2946,21 @@
         <v>12</v>
       </c>
       <c r="G14" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="H14" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="I14" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>162</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>6</v>
@@ -2922,7 +2969,7 @@
         <v>6</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>6</v>
@@ -2931,21 +2978,21 @@
         <v>6</v>
       </c>
       <c r="G15" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="H15" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>183</v>
-      </c>
       <c r="J15" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>6</v>
@@ -2954,7 +3001,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>6</v>
@@ -2963,21 +3010,21 @@
         <v>3</v>
       </c>
       <c r="G16" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="H16" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="I16" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="J16" s="1" t="s">
         <v>186</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>6</v>
@@ -2986,7 +3033,7 @@
         <v>3</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>6</v>
@@ -2995,21 +3042,21 @@
         <v>1</v>
       </c>
       <c r="G17" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="H17" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="H17" s="1" t="s">
+      <c r="I17" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="I17" s="1" t="s">
+      <c r="J17" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="J17" s="3" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>6</v>
@@ -3018,7 +3065,7 @@
         <v>12</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>7</v>
@@ -3027,21 +3074,21 @@
         <v>12</v>
       </c>
       <c r="G18" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="H18" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="I18" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="J18" s="5" t="s">
         <v>194</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>6</v>
@@ -3050,7 +3097,7 @@
         <v>6</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>7</v>
@@ -3059,21 +3106,21 @@
         <v>6</v>
       </c>
       <c r="G19" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="H19" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="H19" s="5" t="s">
+      <c r="I19" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="I19" s="1" t="s">
+      <c r="J19" s="3" t="s">
         <v>198</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>6</v>
@@ -3082,7 +3129,7 @@
         <v>3</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>7</v>
@@ -3091,21 +3138,21 @@
         <v>3</v>
       </c>
       <c r="G20" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="H20" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="H20" s="1" t="s">
+      <c r="I20" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="I20" s="1" t="s">
+      <c r="J20" s="5" t="s">
         <v>202</v>
-      </c>
-      <c r="J20" s="5" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>6</v>
@@ -3114,7 +3161,7 @@
         <v>3</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>7</v>
@@ -3123,21 +3170,21 @@
         <v>1</v>
       </c>
       <c r="G21" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I21" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="H21" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="I21" s="1" t="s">
+      <c r="J21" s="3" t="s">
         <v>205</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>7</v>
@@ -3146,7 +3193,7 @@
         <v>12</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>6</v>
@@ -3155,21 +3202,21 @@
         <v>12</v>
       </c>
       <c r="G22" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="H22" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="H22" s="1" t="s">
+      <c r="I22" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="I22" s="1" t="s">
+      <c r="J22" s="1" t="s">
         <v>214</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>7</v>
@@ -3178,7 +3225,7 @@
         <v>6</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>6</v>
@@ -3187,21 +3234,21 @@
         <v>6</v>
       </c>
       <c r="G23" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="H23" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="H23" s="1" t="s">
+      <c r="I23" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="I23" s="1" t="s">
+      <c r="J23" s="1" t="s">
         <v>218</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>7</v>
@@ -3210,7 +3257,7 @@
         <v>3</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>6</v>
@@ -3219,21 +3266,21 @@
         <v>3</v>
       </c>
       <c r="G24" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="H24" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="H24" s="1" t="s">
+      <c r="I24" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="I24" s="1" t="s">
+      <c r="J24" s="1" t="s">
         <v>222</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>7</v>
@@ -3242,7 +3289,7 @@
         <v>3</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>6</v>
@@ -3251,21 +3298,21 @@
         <v>1</v>
       </c>
       <c r="G25" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H25" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="H25" s="1" t="s">
+      <c r="I25" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="I25" s="1" t="s">
-        <v>226</v>
-      </c>
       <c r="J25" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>7</v>
@@ -3274,7 +3321,7 @@
         <v>12</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>7</v>
@@ -3283,21 +3330,21 @@
         <v>12</v>
       </c>
       <c r="G26" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="H26" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="I26" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="I26" s="1" t="s">
+      <c r="J26" s="5" t="s">
         <v>229</v>
-      </c>
-      <c r="J26" s="5" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>7</v>
@@ -3306,7 +3353,7 @@
         <v>6</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>7</v>
@@ -3315,21 +3362,21 @@
         <v>6</v>
       </c>
       <c r="G27" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="H27" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="H27" s="1" t="s">
+      <c r="I27" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="I27" s="1" t="s">
+      <c r="J27" s="3" t="s">
         <v>233</v>
-      </c>
-      <c r="J27" s="3" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>7</v>
@@ -3338,7 +3385,7 @@
         <v>3</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>7</v>
@@ -3347,21 +3394,21 @@
         <v>3</v>
       </c>
       <c r="G28" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="H28" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H28" s="1" t="s">
+      <c r="I28" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="I28" s="1" t="s">
+      <c r="J28" s="5" t="s">
         <v>237</v>
-      </c>
-      <c r="J28" s="5" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>7</v>
@@ -3370,7 +3417,7 @@
         <v>3</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>7</v>
@@ -3379,16 +3426,16 @@
         <v>1</v>
       </c>
       <c r="G29" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="H29" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="H29" s="1" t="s">
+      <c r="I29" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="I29" s="1" t="s">
+      <c r="J29" s="5" t="s">
         <v>241</v>
-      </c>
-      <c r="J29" s="5" t="s">
-        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -3420,7 +3467,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -3454,22 +3501,22 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>10</v>
@@ -3477,7 +3524,7 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B4" s="4">
         <v>-1190</v>
@@ -3486,13 +3533,13 @@
         <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>16</v>
@@ -3500,7 +3547,7 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -3534,7 +3581,7 @@
         <v>4</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>4</v>
@@ -3542,65 +3589,65 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="I8" s="3" t="s">
         <v>249</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="H9" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="G9" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="H9" s="1" t="s">
+      <c r="I9" s="5" t="s">
         <v>255</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -3614,39 +3661,39 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C13" s="1" t="s">
+      <c r="D13" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="G13" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F13" s="1" t="s">
+      <c r="H13" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="I13" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="G13" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="H13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>6</v>
@@ -3655,7 +3702,7 @@
         <v>12</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>6</v>
@@ -3664,21 +3711,21 @@
         <v>12</v>
       </c>
       <c r="G14" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="H14" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="I14" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="I14" s="1" t="s">
-        <v>259</v>
-      </c>
       <c r="J14" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>6</v>
@@ -3687,7 +3734,7 @@
         <v>6</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>6</v>
@@ -3696,21 +3743,21 @@
         <v>6</v>
       </c>
       <c r="G15" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="H15" s="3" t="s">
         <v>260</v>
       </c>
-      <c r="H15" s="3" t="s">
+      <c r="I15" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="J15" s="1" t="s">
         <v>262</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>6</v>
@@ -3719,7 +3766,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>6</v>
@@ -3728,21 +3775,21 @@
         <v>3</v>
       </c>
       <c r="G16" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="I16" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="H16" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="I16" s="1" t="s">
+      <c r="J16" s="5" t="s">
         <v>265</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>6</v>
@@ -3751,7 +3798,7 @@
         <v>3</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>6</v>
@@ -3760,21 +3807,21 @@
         <v>1</v>
       </c>
       <c r="G17" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="H17" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="I17" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="I17" s="1" t="s">
+      <c r="J17" s="5" t="s">
         <v>269</v>
-      </c>
-      <c r="J17" s="5" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>6</v>
@@ -3783,7 +3830,7 @@
         <v>12</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>7</v>
@@ -3792,21 +3839,21 @@
         <v>12</v>
       </c>
       <c r="G18" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="I18" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="H18" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="I18" s="1" t="s">
+      <c r="J18" s="5" t="s">
         <v>272</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>6</v>
@@ -3815,7 +3862,7 @@
         <v>6</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>7</v>
@@ -3824,21 +3871,21 @@
         <v>6</v>
       </c>
       <c r="G19" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="I19" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="H19" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="I19" s="1" t="s">
+      <c r="J19" s="1" t="s">
         <v>275</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>6</v>
@@ -3847,7 +3894,7 @@
         <v>3</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>7</v>
@@ -3856,21 +3903,21 @@
         <v>3</v>
       </c>
       <c r="G20" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="I20" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="H20" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>278</v>
-      </c>
       <c r="J20" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>6</v>
@@ -3879,7 +3926,7 @@
         <v>3</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>7</v>
@@ -3888,21 +3935,21 @@
         <v>1</v>
       </c>
       <c r="G21" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="H21" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="H21" s="3" t="s">
+      <c r="I21" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="J21" s="5" t="s">
         <v>281</v>
-      </c>
-      <c r="J21" s="5" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>7</v>
@@ -3911,7 +3958,7 @@
         <v>12</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>6</v>
@@ -3923,18 +3970,18 @@
         <v>-1339</v>
       </c>
       <c r="H22" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="I22" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="I22" s="1" t="s">
+      <c r="J22" s="5" t="s">
         <v>284</v>
-      </c>
-      <c r="J22" s="5" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>7</v>
@@ -3943,7 +3990,7 @@
         <v>6</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>6</v>
@@ -3952,21 +3999,21 @@
         <v>6</v>
       </c>
       <c r="G23" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="H23" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="H23" s="1" t="s">
+      <c r="I23" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="I23" s="1" t="s">
+      <c r="J23" s="3" t="s">
         <v>288</v>
-      </c>
-      <c r="J23" s="3" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>7</v>
@@ -3975,7 +4022,7 @@
         <v>3</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>6</v>
@@ -3984,21 +4031,21 @@
         <v>3</v>
       </c>
       <c r="G24" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="H24" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="H24" s="1" t="s">
+      <c r="I24" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="I24" s="1" t="s">
-        <v>292</v>
-      </c>
       <c r="J24" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>7</v>
@@ -4007,7 +4054,7 @@
         <v>3</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>6</v>
@@ -4016,21 +4063,21 @@
         <v>1</v>
       </c>
       <c r="G25" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="H25" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="H25" s="1" t="s">
+      <c r="I25" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="J25" s="3" t="s">
         <v>294</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="J25" s="3" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>7</v>
@@ -4039,7 +4086,7 @@
         <v>12</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>7</v>
@@ -4051,18 +4098,18 @@
         <v>-1519</v>
       </c>
       <c r="H26" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="I26" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="I26" s="1" t="s">
-        <v>297</v>
-      </c>
       <c r="J26" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>7</v>
@@ -4071,7 +4118,7 @@
         <v>6</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>7</v>
@@ -4080,21 +4127,21 @@
         <v>6</v>
       </c>
       <c r="G27" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I27" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="H27" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="I27" s="1" t="s">
+      <c r="J27" s="1" t="s">
         <v>299</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>7</v>
@@ -4103,7 +4150,7 @@
         <v>3</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>7</v>
@@ -4112,21 +4159,21 @@
         <v>3</v>
       </c>
       <c r="G28" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="H28" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="H28" s="1" t="s">
+      <c r="I28" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="I28" s="1" t="s">
-        <v>303</v>
-      </c>
       <c r="J28" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>7</v>
@@ -4135,7 +4182,7 @@
         <v>3</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>7</v>
@@ -4144,16 +4191,16 @@
         <v>1</v>
       </c>
       <c r="G29" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="H29" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="H29" s="1" t="s">
+      <c r="I29" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="I29" s="1" t="s">
+      <c r="J29" s="5" t="s">
         <v>306</v>
-      </c>
-      <c r="J29" s="5" t="s">
-        <v>307</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
estatisticas descritivas - cambio
</commit_message>
<xml_diff>
--- a/graficos_tabelas/preliminares/Tabela_resumo_thetas.xlsx
+++ b/graficos_tabelas/preliminares/Tabela_resumo_thetas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6e8fc6e241c731ae/UFABC/Dissertação/volatilidade-IBOV-GPR/Impacto-geopolitico-ibovespa/graficos_tabelas/preliminares/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="733" documentId="11_F25DC773A252ABDACC1048C0F11B46C65ADE58EB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8DF6CF67-1D4A-4C76-8214-2BB80FD9C855}"/>
+  <xr:revisionPtr revIDLastSave="741" documentId="11_F25DC773A252ABDACC1048C0F11B46C65ADE58EB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA90C009-D415-4793-97EE-E54441718FA4}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="320">
   <si>
     <t>Garch-Midas nos retornos do Ibovespa</t>
   </si>
@@ -976,6 +976,18 @@
   </si>
   <si>
     <t>0.226</t>
+  </si>
+  <si>
+    <t>0.354</t>
+  </si>
+  <si>
+    <t>0.372</t>
+  </si>
+  <si>
+    <t>0.542</t>
+  </si>
+  <si>
+    <t>LOG-DIFF (CAMBIO)</t>
   </si>
 </sst>
 </file>
@@ -1076,6 +1088,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1084,9 +1099,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1403,15 +1415,15 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -1521,15 +1533,15 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
@@ -1624,15 +1636,15 @@
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
@@ -1771,18 +1783,18 @@
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
@@ -2369,15 +2381,15 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -2449,15 +2461,15 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -2529,15 +2541,15 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
@@ -2570,19 +2582,19 @@
         <v>48</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>10</v>
+        <v>167</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>49</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>10</v>
+        <v>257</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>51</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -2593,31 +2605,31 @@
         <v>-1190</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>67</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>16</v>
+        <v>317</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>68</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>16</v>
+        <v>318</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
@@ -2717,15 +2729,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -2797,17 +2809,17 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -2869,7 +2881,7 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>149</v>
+        <v>319</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -2881,18 +2893,18 @@
       <c r="I9" s="1"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
@@ -3466,15 +3478,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -3507,19 +3519,19 @@
         <v>48</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>10</v>
+        <v>167</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>49</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>10</v>
+        <v>257</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>51</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>10</v>
+        <v>294</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -3530,33 +3542,33 @@
         <v>-1190</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>16</v>
+        <v>316</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>67</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>16</v>
+        <v>317</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>68</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>16</v>
+        <v>318</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="8" t="s">
         <v>242</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -3646,18 +3658,18 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
@@ -3966,7 +3978,7 @@
       <c r="F22" s="1">
         <v>12</v>
       </c>
-      <c r="G22" s="9">
+      <c r="G22" s="6">
         <v>-1339</v>
       </c>
       <c r="H22" s="1" t="s">
@@ -4094,7 +4106,7 @@
       <c r="F26" s="1">
         <v>12</v>
       </c>
-      <c r="G26" s="9">
+      <c r="G26" s="6">
         <v>-1519</v>
       </c>
       <c r="H26" s="1" t="s">

</xml_diff>